<commit_message>
Add CLM diagnosis interview protocol and route choice
</commit_message>
<xml_diff>
--- a/technologies/06_CLM/30 Документация/20 Сессия/Управление_Директорами_CLM_Продукт_02_Сессия_рабочая_книга_V1.xlsx
+++ b/technologies/06_CLM/30 Документация/20 Сессия/Управление_Директорами_CLM_Продукт_02_Сессия_рабочая_книга_V1.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:workbookPr/>
   <x:workbookProtection/>
   <x:bookViews>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="0"/>
-  <x:fonts count="4">
+  <x:fonts count="6">
     <x:font>
       <x:name val="Calibri"/>
       <x:family val="2"/>
@@ -44,6 +44,20 @@
       <x:b val="1"/>
       <x:color rgb="0016324F"/>
       <x:sz val="12"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+      <x:family xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="2"/>
+      <x:scheme xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="minor"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color theme="1"/>
+      <x:name val="Arial"/>
+      <x:family xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="2"/>
+      <x:scheme xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="minor"/>
     </x:font>
   </x:fonts>
   <x:fills count="5">
@@ -95,7 +109,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -112,6 +126,21 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyFill="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1054,7 +1083,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
     <x:pageSetUpPr/>
@@ -1063,8 +1092,8 @@
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22" customWidth="1"/>
-    <x:col min="2" max="2" width="22" customWidth="1"/>
-    <x:col min="3" max="3" width="22" customWidth="1"/>
+    <x:col min="2" max="2" width="36" customWidth="1"/>
+    <x:col min="3" max="3" width="10" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1129,14 +1158,17 @@
       <x:c r="B6" s="4" t="inlineStr"/>
       <x:c r="C6" s="4" t="inlineStr"/>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="6" t="str">
+    <x:row r="7" ht="72" customHeight="1">
+      <x:c r="A7" s="10" t="str">
         <x:v>Решение перехода</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="str">
-        <x:v>SPRINT — паспорт полный; HOLD — доработка в Сессии; STOP — обязательный блокер</x:v>
+      <x:c r="B7" s="10" t="str">
+        <x:v>КОНСУЛЬТАНТ — полный Паспорт
+КЛИЕНТ — самостоятельная реализация по Паспорту
+HOLD — доработка в Сессии
+STOP — обязательный блокер</x:v>
       </x:c>
-      <x:c r="C7" s="3" t="n"/>
+      <x:c r="C7" s="11" t="n"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>